<commit_message>
updated summary analysis, adding summary of dosing data (number of larvae dosed in F0 for each treatment and lineage).
</commit_message>
<xml_diff>
--- a/raw_data/performance_data.xlsx
+++ b/raw_data/performance_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joegunn/Desktop/Projects/active_projects/CPB_Phenotype/raw_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joegunn/Desktop/projects/active_projects/CPB_Phenotype/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BFE6BB-2BAE-714F-B45C-E8CB9B01325F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BF4ACAD-32E2-9645-97E1-034A4487C57F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26040" yWindow="960" windowWidth="25040" windowHeight="16940" xr2:uid="{95B528D8-456B-7F43-840E-A5E8A7FC98F5}"/>
+    <workbookView xWindow="41760" yWindow="500" windowWidth="25040" windowHeight="16940" xr2:uid="{95B528D8-456B-7F43-840E-A5E8A7FC98F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2425,6 +2425,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA7E2E4-25E3-F34B-8586-39E393485815}">
   <dimension ref="A1:BK420"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:63" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>